<commit_message>
Tab 1 Financials: Handled with full precision, absolute (positive) variance columns, and a clean Excel export.
Tab 2 Aggregation: Automatically merges multiple rows from Sheet 1 if they belong to the same product and channel.

Tab 2 Guardrails: Automatically skips any summary or total row in Sheet 2 that doesn't have a specific Cost Type in Column C.

Product Filter: High-speed filtering by drug name for focused auditing.
</commit_message>
<xml_diff>
--- a/sample files for test/row_rise_data.xlsx
+++ b/sample files for test/row_rise_data.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet2" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="34">
   <si>
     <t xml:space="preserve">Currency</t>
   </si>
@@ -98,6 +98,30 @@
   </si>
   <si>
     <t xml:space="preserve">PROMOTIONAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ONCOLOGY &amp; HEMATOLOGY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLUMVI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EVRYSDI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POLIVY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TECENTRIQ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BREAST CANCER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HEPATOCELLULAR CARCINOMA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LUNG CANCER</t>
   </si>
 </sst>
 </file>
@@ -107,7 +131,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -141,13 +165,6 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="&quot;Google Sans Text&quot;"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -194,15 +211,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -215,11 +224,11 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -232,31 +241,6 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF1F1F1F"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -495,266 +479,1068 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Z1048576"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.87"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="7.81"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="29.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="33.06"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="15.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="20.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="21.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="13.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="16.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="16.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="25.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="14.96"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="17" style="2" width="11.53"/>
-  </cols>
+  <dimension ref="A1:P21"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="4" t="s">
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="5"/>
-      <c r="R1" s="5"/>
-      <c r="S1" s="5"/>
-      <c r="T1" s="5"/>
-      <c r="U1" s="5"/>
-      <c r="V1" s="5"/>
-      <c r="W1" s="5"/>
-      <c r="X1" s="5"/>
-      <c r="Y1" s="5"/>
-      <c r="Z1" s="5"/>
-    </row>
-    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" s="6" t="n">
-        <v>2025</v>
-      </c>
-      <c r="C2" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="F2" s="6" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="I2" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="J2" s="6" t="s">
+      <c r="I2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J2" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K2" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="L2" s="6" t="n">
+      <c r="L2" s="3" t="n">
         <v>12795737.46</v>
       </c>
-      <c r="M2" s="6" t="n">
+      <c r="M2" s="3" t="n">
         <v>8170741.85</v>
       </c>
-      <c r="N2" s="6" t="n">
+      <c r="N2" s="3" t="n">
         <v>41440010.93</v>
       </c>
-      <c r="O2" s="6" t="n">
+      <c r="O2" s="3" t="n">
         <v>34229300.96</v>
       </c>
-      <c r="P2" s="6" t="n">
+      <c r="P2" s="3" t="n">
         <v>4.189252529</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="6" t="n">
-        <v>2025</v>
-      </c>
-      <c r="C3" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="6" t="s">
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="J3" s="6" t="s">
+      <c r="I3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="K3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="L3" s="6" t="n">
+      <c r="L3" s="3" t="n">
         <v>2214208.42</v>
       </c>
-      <c r="M3" s="6" t="n">
+      <c r="M3" s="3" t="n">
         <v>3099891.788</v>
       </c>
-      <c r="N3" s="6" t="n">
+      <c r="N3" s="3" t="n">
         <v>37261137.35</v>
       </c>
-      <c r="O3" s="6" t="n">
+      <c r="O3" s="3" t="n">
         <v>41099709.11</v>
       </c>
-      <c r="P3" s="6" t="n">
+      <c r="P3" s="3" t="n">
         <v>13.25843349</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="6" t="n">
-        <v>2025</v>
-      </c>
-      <c r="C4" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="6" t="s">
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="J4" s="6" t="s">
+      <c r="I4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="K4" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="L4" s="6" t="n">
-        <v>2506572.5</v>
-      </c>
-      <c r="M4" s="6" t="n">
+      <c r="L4" s="3" t="n">
+        <v>1253286.25</v>
+      </c>
+      <c r="M4" s="3" t="n">
         <v>3307224.443</v>
       </c>
-      <c r="N4" s="6" t="n">
+      <c r="N4" s="3" t="n">
         <v>20881575.16</v>
       </c>
-      <c r="O4" s="6" t="n">
+      <c r="O4" s="3" t="n">
         <v>23219845.82</v>
       </c>
-      <c r="P4" s="6" t="n">
+      <c r="P4" s="3" t="n">
         <v>7.020946482</v>
       </c>
     </row>
-    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>1253286.25</v>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>3307224.443</v>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>20881575.16</v>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>23219845.82</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>7.020946482</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>6092430.08</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>3655458.048</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>8392167.62</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>6427566.202</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>1.758347686</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="L7" s="4" t="n">
+        <v>28350.54</v>
+      </c>
+      <c r="M7" s="4" t="n">
+        <v>39690.756</v>
+      </c>
+      <c r="N7" s="4" t="n">
+        <v>2330560.31</v>
+      </c>
+      <c r="O7" s="4" t="n">
+        <v>2537721.226</v>
+      </c>
+      <c r="P7" s="4" t="n">
+        <v>63.9373366</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>485593.76</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>291356.256</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>1440791.74</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>1194097.096</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>4.098408981</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>1772199.88</v>
+      </c>
+      <c r="M9" s="4" t="n">
+        <v>2481079.832</v>
+      </c>
+      <c r="N9" s="4" t="n">
+        <v>44196082.23</v>
+      </c>
+      <c r="O9" s="4" t="n">
+        <v>48340263.6</v>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>19.48355832</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>301727.88</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>422419.032</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>5210988.05</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>5794223.453</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>13.71676703</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>1304812.98</v>
+      </c>
+      <c r="M11" s="4" t="n">
+        <v>1328173.179</v>
+      </c>
+      <c r="N11" s="4" t="n">
+        <v>5070164.62</v>
+      </c>
+      <c r="O11" s="4" t="n">
+        <v>5120289.967</v>
+      </c>
+      <c r="P11" s="4" t="n">
+        <v>3.855137302</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>3019531.17</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>4227343.638</v>
+      </c>
+      <c r="N12" s="4" t="n">
+        <v>27945439.9</v>
+      </c>
+      <c r="O12" s="4" t="n">
+        <v>31911689.86</v>
+      </c>
+      <c r="P12" s="4" t="n">
+        <v>7.548875273</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="L13" s="4" t="n">
+        <v>28350.54</v>
+      </c>
+      <c r="M13" s="4" t="n">
+        <v>39690.756</v>
+      </c>
+      <c r="N13" s="4" t="n">
+        <v>14102663.62</v>
+      </c>
+      <c r="O13" s="4" t="n">
+        <v>15686460.3</v>
+      </c>
+      <c r="P13" s="4" t="n">
+        <v>395.2169693</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>762777.17</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>880651.2412</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>3412780.32</v>
+      </c>
+      <c r="O14" s="4" t="n">
+        <v>3677449.964</v>
+      </c>
+      <c r="P14" s="4" t="n">
+        <v>4.175830104</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="L15" s="4" t="n">
+        <v>7834638.3</v>
+      </c>
+      <c r="M15" s="4" t="n">
+        <v>6615273.907</v>
+      </c>
+      <c r="N15" s="4" t="n">
+        <v>38045514.83</v>
+      </c>
+      <c r="O15" s="4" t="n">
+        <v>35788830.17</v>
+      </c>
+      <c r="P15" s="4" t="n">
+        <v>5.410029981</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>8751.87</v>
+      </c>
+      <c r="M16" s="4" t="n">
+        <v>12252.618</v>
+      </c>
+      <c r="N16" s="4" t="n">
+        <v>642642.12</v>
+      </c>
+      <c r="O16" s="4" t="n">
+        <v>668186.7502</v>
+      </c>
+      <c r="P16" s="4" t="n">
+        <v>54.53420242</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L17" s="4" t="n">
+        <v>8571.12</v>
+      </c>
+      <c r="M17" s="4" t="n">
+        <v>9765.286467</v>
+      </c>
+      <c r="N17" s="4" t="n">
+        <v>22507.9</v>
+      </c>
+      <c r="O17" s="4" t="n">
+        <v>25356.48964</v>
+      </c>
+      <c r="P17" s="4" t="n">
+        <v>2.596594553</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="L18" s="4" t="n">
+        <v>219251.4</v>
+      </c>
+      <c r="M18" s="4" t="n">
+        <v>270318.4054</v>
+      </c>
+      <c r="N18" s="4" t="n">
+        <v>1589849.55</v>
+      </c>
+      <c r="O18" s="4" t="n">
+        <v>1710725.288</v>
+      </c>
+      <c r="P18" s="4" t="n">
+        <v>6.32855645</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L19" s="4" t="n">
+        <v>356750.79</v>
+      </c>
+      <c r="M19" s="4" t="n">
+        <v>246981.4965</v>
+      </c>
+      <c r="N19" s="4" t="n">
+        <v>892123.07</v>
+      </c>
+      <c r="O19" s="4" t="n">
+        <v>733934.0955</v>
+      </c>
+      <c r="P19" s="4" t="n">
+        <v>2.971615712</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>382593.17</v>
+      </c>
+      <c r="M20" s="4" t="n">
+        <v>535630.438</v>
+      </c>
+      <c r="N20" s="4" t="n">
+        <v>14327802.23</v>
+      </c>
+      <c r="O20" s="4" t="n">
+        <v>15601384.65</v>
+      </c>
+      <c r="P20" s="4" t="n">
+        <v>29.12714353</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L21" s="4" t="n">
+        <v>1958892.37</v>
+      </c>
+      <c r="M21" s="4" t="n">
+        <v>1175335.422</v>
+      </c>
+      <c r="N21" s="4" t="n">
+        <v>4204124.16</v>
+      </c>
+      <c r="O21" s="4" t="n">
+        <v>3248314.018</v>
+      </c>
+      <c r="P21" s="4" t="n">
+        <v>2.763733618</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>